<commit_message>
updated source-sink manipulation scripts
</commit_message>
<xml_diff>
--- a/Data/2022_Carb_data/Stem_all_additional_analysis.xlsx
+++ b/Data/2022_Carb_data/Stem_all_additional_analysis.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ximinpiao/Documents/GitHub/UTR-Soybean-BioCro/Data/2022_Carb_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A7AD9194-607F-4843-88FD-27DFF0D56160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2696B45-917C-7A4C-B6C8-9400743A961C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4880" yWindow="-14520" windowWidth="26880" windowHeight="14520" activeTab="2" xr2:uid="{3D71B5A5-8708-C847-A3C0-BE85470492FC}"/>
+    <workbookView xWindow="1880" yWindow="1780" windowWidth="26880" windowHeight="14520" activeTab="1" xr2:uid="{3D71B5A5-8708-C847-A3C0-BE85470492FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Stem_all" sheetId="1" r:id="rId1"/>
     <sheet name="C" sheetId="2" r:id="rId2"/>
     <sheet name="DM" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="40">
   <si>
     <t>Sample ID</t>
   </si>
@@ -153,13 +154,16 @@
   <si>
     <t>Total_std</t>
   </si>
+  <si>
+    <t>Starch%</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -663,24 +667,25 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="33" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="34" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="35" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="36" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -1154,7 +1159,8 @@
         <v>186</v>
       </c>
       <c r="D2">
-        <v>11</v>
+        <f>HOUR(B2)</f>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>186.45833300000001</v>
@@ -1237,7 +1243,8 @@
         <v>186</v>
       </c>
       <c r="D3">
-        <v>14</v>
+        <f t="shared" ref="D3:D18" si="0">HOUR(B3)</f>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>186.58333300000001</v>
@@ -1320,7 +1327,8 @@
         <v>186</v>
       </c>
       <c r="D4">
-        <v>17</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>186.70833300000001</v>
@@ -1403,7 +1411,8 @@
         <v>186</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>186.83333300000001</v>
@@ -1486,7 +1495,8 @@
         <v>186</v>
       </c>
       <c r="D6">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="E6">
         <v>186.95833300000001</v>
@@ -1569,7 +1579,8 @@
         <v>187</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="E7">
         <v>187.08333300000001</v>
@@ -1652,7 +1663,8 @@
         <v>187</v>
       </c>
       <c r="D8">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>4</v>
       </c>
       <c r="E8">
         <v>187.20833300000001</v>
@@ -1735,7 +1747,8 @@
         <v>187</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="E9">
         <v>187.33333300000001</v>
@@ -1818,7 +1831,8 @@
         <v>209</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="E10">
         <v>209.33333300000001</v>
@@ -1901,6 +1915,7 @@
         <v>209</v>
       </c>
       <c r="D11">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="E11">
@@ -1984,7 +1999,8 @@
         <v>236</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="E12">
         <v>236.33333300000001</v>
@@ -2067,6 +2083,7 @@
         <v>236</v>
       </c>
       <c r="D13">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="E13">
@@ -2150,7 +2167,8 @@
         <v>236</v>
       </c>
       <c r="D14">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="E14">
         <v>236.83333300000001</v>
@@ -2233,7 +2251,8 @@
         <v>258</v>
       </c>
       <c r="D15">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="E15">
         <v>258.33333299999998</v>
@@ -2316,6 +2335,7 @@
         <v>258</v>
       </c>
       <c r="D16">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="E16">
@@ -2399,7 +2419,8 @@
         <v>258</v>
       </c>
       <c r="D17">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="E17">
         <v>258.83333299999998</v>
@@ -2482,6 +2503,7 @@
         <v>278</v>
       </c>
       <c r="D18">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="E18">
@@ -2763,7 +2785,7 @@
         <v>2.298</v>
       </c>
       <c r="AB2" s="5">
-        <f t="shared" ref="AB2:AB18" si="1">SQRT((((H2-$Z2)^2)*T2+((J2-$Z2)^2)*U2+((L2-$Z2)^2)*V2+((N2-$Z2)^2)*W2)/(X2-1))</f>
+        <f t="shared" ref="AB2:AB17" si="1">SQRT((((H2-$Z2)^2)*T2+((J2-$Z2)^2)*U2+((L2-$Z2)^2)*V2+((N2-$Z2)^2)*W2)/(X2-1))</f>
         <v>0.7515772207221797</v>
       </c>
       <c r="AC2" s="6">
@@ -2784,7 +2806,7 @@
       </c>
       <c r="AH2" s="5">
         <f>((H2+I2-$AD$19)^2)*T2+((J2+K2-$AD$19)^2)*U2+((L2+M2-$AD$19)^2)*V2+((N2+O2-$AD$19)^2)*W2</f>
-        <v>13.030629661669924</v>
+        <v>12.679427723278547</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.2">
@@ -2906,7 +2928,7 @@
       </c>
       <c r="AH3" s="5">
         <f t="shared" ref="AH3:AH18" si="8">((H3+I3-$AD$19)^2)*T3+((J3+K3-$AD$19)^2)*U3+((L3+M3-$AD$19)^2)*V3+((N3+O3-$AD$19)^2)*W3</f>
-        <v>2.0308741286132821</v>
+        <v>1.9762320672837372</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.2">
@@ -3028,7 +3050,7 @@
       </c>
       <c r="AH4" s="5">
         <f t="shared" si="8"/>
-        <v>0.78886991416992214</v>
+        <v>0.85321208327854736</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.2">
@@ -3150,7 +3172,7 @@
       </c>
       <c r="AH5" s="5">
         <f t="shared" si="8"/>
-        <v>1.5573665379199217</v>
+        <v>1.7484303621020774</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.2">
@@ -3272,7 +3294,7 @@
       </c>
       <c r="AH6" s="5">
         <f t="shared" si="8"/>
-        <v>0.89217403347656243</v>
+        <v>0.70648525809688434</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.2">
@@ -3394,7 +3416,7 @@
       </c>
       <c r="AH7" s="5">
         <f t="shared" si="8"/>
-        <v>7.347778752919921</v>
+        <v>7.0691219244550147</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.2">
@@ -3516,7 +3538,7 @@
       </c>
       <c r="AH8" s="5">
         <f t="shared" si="8"/>
-        <v>5.1371192379199222</v>
+        <v>5.3156038115138422</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.2">
@@ -3638,7 +3660,7 @@
       </c>
       <c r="AH9" s="5">
         <f t="shared" si="8"/>
-        <v>10.64130058722656</v>
+        <v>11.405130812214534</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.2">
@@ -3760,7 +3782,7 @@
       </c>
       <c r="AH10" s="5">
         <f t="shared" si="8"/>
-        <v>43.82801102847656</v>
+        <v>42.720892147508636</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.2">
@@ -3882,7 +3904,7 @@
       </c>
       <c r="AH11" s="5">
         <f t="shared" si="8"/>
-        <v>18.800914190976574</v>
+        <v>17.96124733103807</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.2">
@@ -4004,7 +4026,7 @@
       </c>
       <c r="AH12" s="5">
         <f t="shared" si="8"/>
-        <v>1.2717395791699215</v>
+        <v>1.497038977396195</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.2">
@@ -4126,7 +4148,7 @@
       </c>
       <c r="AH13" s="5">
         <f t="shared" si="8"/>
-        <v>0.35311995166992094</v>
+        <v>0.48393202445501715</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.2">
@@ -4248,7 +4270,7 @@
       </c>
       <c r="AH14" s="5">
         <f t="shared" si="8"/>
-        <v>1.6575771616699209</v>
+        <v>1.8015402691608997</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.2">
@@ -4370,7 +4392,7 @@
       </c>
       <c r="AH15" s="5">
         <f t="shared" si="8"/>
-        <v>4.0251166891699208</v>
+        <v>4.1595024126903111</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.2">
@@ -4492,7 +4514,7 @@
       </c>
       <c r="AH16" s="5">
         <f t="shared" si="8"/>
-        <v>2.9178982098632789</v>
+        <v>2.6687780755190276</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.2">
@@ -4614,7 +4636,7 @@
       </c>
       <c r="AH17" s="5">
         <f t="shared" si="8"/>
-        <v>0.29999934861328104</v>
+        <v>0.27165935669550145</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.2">
@@ -4736,17 +4758,17 @@
       </c>
       <c r="AH18" s="5">
         <f t="shared" si="8"/>
-        <v>6.2663387893066389</v>
+        <v>6.5680795183477514</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.2">
       <c r="AD19" s="14">
-        <f>AVERAGE(AD3:AD18)</f>
-        <v>2.5908656249999997</v>
+        <f>AVERAGE(AD2:AD18)</f>
+        <v>2.6504264705882354</v>
       </c>
       <c r="AH19" s="5">
-        <f>SQRT(SUM(AH2:AH17)/(SUM(X2:X17)-1))</f>
-        <v>1.5450221749590238</v>
+        <f>SQRT(SUM(AH2:AH18)/(SUM(X2:X17)-1))</f>
+        <v>1.580389681343356</v>
       </c>
     </row>
   </sheetData>
@@ -4958,7 +4980,7 @@
         <v>68.94</v>
       </c>
       <c r="AB2" s="5">
-        <f t="shared" ref="AB2:AB18" si="1">SQRT((((H2-$Z2)^2)*T2+((J2-$Z2)^2)*U2+((L2-$Z2)^2)*V2+((N2-$Z2)^2)*W2)/(X2-1))</f>
+        <f t="shared" ref="AB2:AB17" si="1">SQRT((((H2-$Z2)^2)*T2+((J2-$Z2)^2)*U2+((L2-$Z2)^2)*V2+((N2-$Z2)^2)*W2)/(X2-1))</f>
         <v>22.547316621665381</v>
       </c>
       <c r="AC2" s="6">
@@ -4979,7 +5001,7 @@
       </c>
       <c r="AH2" s="5">
         <f>((H2+I2-$AD$19)^2)*T2+((J2+K2-$AD$19)^2)*U2+((L2+M2-$AD$19)^2)*V2+((N2+O2-$AD$19)^2)*W2</f>
-        <v>11727.566695502928</v>
+        <v>11411.484950950691</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.2">
@@ -5101,7 +5123,7 @@
       </c>
       <c r="AH3" s="5">
         <f t="shared" ref="AH3:AH18" si="8">((H3+I3-$AD$19)^2)*T3+((J3+K3-$AD$19)^2)*U3+((L3+M3-$AD$19)^2)*V3+((N3+O3-$AD$19)^2)*W3</f>
-        <v>1827.7867157519529</v>
+        <v>1778.6088605553632</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.2">
@@ -5223,7 +5245,7 @@
       </c>
       <c r="AH4" s="5">
         <f t="shared" si="8"/>
-        <v>709.98292275293034</v>
+        <v>767.89087495069259</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.2">
@@ -5345,7 +5367,7 @@
       </c>
       <c r="AH5" s="5">
         <f t="shared" si="8"/>
-        <v>1401.6298841279304</v>
+        <v>1573.5873258918691</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.2">
@@ -5467,7 +5489,7 @@
       </c>
       <c r="AH6" s="5">
         <f t="shared" si="8"/>
-        <v>802.95663012890509</v>
+        <v>635.8367322871967</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.2">
@@ -5589,7 +5611,7 @@
       </c>
       <c r="AH7" s="5">
         <f t="shared" si="8"/>
-        <v>6613.0008776279246</v>
+        <v>6362.2097320095118</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.2">
@@ -5711,7 +5733,7 @@
       </c>
       <c r="AH8" s="5">
         <f t="shared" si="8"/>
-        <v>4623.4073141279314</v>
+        <v>4784.0434303624579</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.2">
@@ -5833,7 +5855,7 @@
       </c>
       <c r="AH9" s="5">
         <f t="shared" si="8"/>
-        <v>9577.1705285039079</v>
+        <v>10264.617730993081</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.2">
@@ -5955,7 +5977,7 @@
       </c>
       <c r="AH10" s="5">
         <f t="shared" si="8"/>
-        <v>39445.2099256289</v>
+        <v>38448.80293275779</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.2">
@@ -6077,7 +6099,7 @@
       </c>
       <c r="AH11" s="5">
         <f t="shared" si="8"/>
-        <v>16920.822771878902</v>
+        <v>16165.122597934254</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.2">
@@ -6199,7 +6221,7 @@
       </c>
       <c r="AH12" s="5">
         <f t="shared" si="8"/>
-        <v>1144.5656212529311</v>
+        <v>1347.3350796565751</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.2">
@@ -6321,7 +6343,7 @@
       </c>
       <c r="AH13" s="5">
         <f t="shared" si="8"/>
-        <v>317.8079565029301</v>
+        <v>435.53882200951568</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.2">
@@ -6443,7 +6465,7 @@
       </c>
       <c r="AH14" s="5">
         <f t="shared" si="8"/>
-        <v>1491.8194455029306</v>
+        <v>1621.3862422448101</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.2">
@@ -6565,7 +6587,7 @@
       </c>
       <c r="AH15" s="5">
         <f t="shared" si="8"/>
-        <v>3622.6050202529304</v>
+        <v>3743.5521714212809</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.2">
@@ -6687,7 +6709,7 @@
       </c>
       <c r="AH16" s="5">
         <f t="shared" si="8"/>
-        <v>2626.1083888769499</v>
+        <v>2401.9002679671257</v>
       </c>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.2">
@@ -6809,7 +6831,7 @@
       </c>
       <c r="AH17" s="5">
         <f t="shared" si="8"/>
-        <v>269.999413751953</v>
+        <v>244.49342102595153</v>
       </c>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.2">
@@ -6931,17 +6953,630 @@
       </c>
       <c r="AH18" s="5">
         <f t="shared" si="8"/>
-        <v>5639.7049103759773</v>
+        <v>5911.2715665129763</v>
       </c>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.2">
       <c r="AD19" s="14">
-        <f>AVERAGE(AD3:AD18)</f>
-        <v>77.725968750000007</v>
+        <f>AVERAGE(AD2:AD18)</f>
+        <v>79.512794117647061</v>
       </c>
       <c r="AH19" s="5">
-        <f>SQRT(SUM(AH2:AH17)/(SUM(X2:X17)-1))</f>
-        <v>46.35066524877071</v>
+        <f>SQRT(SUM(AH2:AH18)/(SUM(X2:X17)-1))</f>
+        <v>47.411690440300681</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03FD6867-1FD2-4047-BA21-C7CAA1AA11A7}">
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" customWidth="1"/>
+    <col min="6" max="6" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>39.161999999999999</v>
+      </c>
+      <c r="D2">
+        <v>53.97110026671681</v>
+      </c>
+      <c r="E2" s="17">
+        <f>C2/I2</f>
+        <v>0.36226896819670307</v>
+      </c>
+      <c r="F2">
+        <v>68.94</v>
+      </c>
+      <c r="G2">
+        <v>22.547316621665381</v>
+      </c>
+      <c r="H2" s="17">
+        <v>0.63773103180329682</v>
+      </c>
+      <c r="I2">
+        <v>108.102</v>
+      </c>
+      <c r="J2">
+        <v>66.930773460344824</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>23.625</v>
+      </c>
+      <c r="D3">
+        <v>13.758883748327841</v>
+      </c>
+      <c r="E3" s="17">
+        <f t="shared" ref="E3:E18" si="0">C3/I3</f>
+        <v>0.27631578947368424</v>
+      </c>
+      <c r="F3">
+        <v>61.875</v>
+      </c>
+      <c r="G3">
+        <v>73.414247502026868</v>
+      </c>
+      <c r="H3" s="17">
+        <v>0.72368421052631582</v>
+      </c>
+      <c r="I3">
+        <v>85.5</v>
+      </c>
+      <c r="J3">
+        <v>41.314835011167595</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>23.963999999999999</v>
+      </c>
+      <c r="D4">
+        <v>14.460178007203094</v>
+      </c>
+      <c r="E4" s="17">
+        <f t="shared" si="0"/>
+        <v>0.32729656641809396</v>
+      </c>
+      <c r="F4">
+        <v>49.253999999999998</v>
+      </c>
+      <c r="G4">
+        <v>46.060204486081652</v>
+      </c>
+      <c r="H4" s="17">
+        <v>0.67270343358190621</v>
+      </c>
+      <c r="I4">
+        <v>73.217999999999989</v>
+      </c>
+      <c r="J4">
+        <v>18.014127455971888</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>23.411999999999995</v>
+      </c>
+      <c r="D5">
+        <v>14.985000900900873</v>
+      </c>
+      <c r="E5" s="17">
+        <f t="shared" si="0"/>
+        <v>0.37411313518696065</v>
+      </c>
+      <c r="F5">
+        <v>39.167999999999999</v>
+      </c>
+      <c r="G5">
+        <v>29.952585066076413</v>
+      </c>
+      <c r="H5" s="17">
+        <v>0.62588686481303935</v>
+      </c>
+      <c r="I5">
+        <v>62.58</v>
+      </c>
+      <c r="J5">
+        <v>18.886884020398913</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>59.152499999999996</v>
+      </c>
+      <c r="D6">
+        <v>15.331339961007975</v>
+      </c>
+      <c r="E6" s="17">
+        <f t="shared" si="0"/>
+        <v>0.65499028352184963</v>
+      </c>
+      <c r="F6">
+        <v>31.157999999999998</v>
+      </c>
+      <c r="G6">
+        <v>26.281982370433344</v>
+      </c>
+      <c r="H6" s="17">
+        <v>0.34500971647815037</v>
+      </c>
+      <c r="I6">
+        <v>90.31049999999999</v>
+      </c>
+      <c r="J6">
+        <v>7.516092136210144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>52.325999999999993</v>
+      </c>
+      <c r="D7">
+        <v>42.188256233222049</v>
+      </c>
+      <c r="E7" s="17">
+        <f t="shared" si="0"/>
+        <v>0.5129396541583342</v>
+      </c>
+      <c r="F7">
+        <v>49.686</v>
+      </c>
+      <c r="G7">
+        <v>14.740300349327567</v>
+      </c>
+      <c r="H7" s="17">
+        <v>0.48706034584166569</v>
+      </c>
+      <c r="I7">
+        <v>102.012</v>
+      </c>
+      <c r="J7">
+        <v>49.211619237736919</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>9.9659999999999993</v>
+      </c>
+      <c r="D8">
+        <v>12.471471605227666</v>
+      </c>
+      <c r="E8" s="17">
+        <f t="shared" si="0"/>
+        <v>0.15660946633980766</v>
+      </c>
+      <c r="F8">
+        <v>53.669999999999995</v>
+      </c>
+      <c r="G8">
+        <v>60.181358582556889</v>
+      </c>
+      <c r="H8" s="17">
+        <v>0.84339053366019234</v>
+      </c>
+      <c r="I8">
+        <v>63.635999999999996</v>
+      </c>
+      <c r="J8">
+        <v>44.87664011487491</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>9.400500000000001</v>
+      </c>
+      <c r="D9">
+        <v>5.9053420730724824</v>
+      </c>
+      <c r="E9" s="17">
+        <f t="shared" si="0"/>
+        <v>0.30793042452830194</v>
+      </c>
+      <c r="F9">
+        <v>21.127499999999998</v>
+      </c>
+      <c r="G9">
+        <v>20.628053800664187</v>
+      </c>
+      <c r="H9" s="17">
+        <v>0.69206957547169812</v>
+      </c>
+      <c r="I9">
+        <v>30.527999999999999</v>
+      </c>
+      <c r="J9">
+        <v>14.906123037195151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>7.6896876399500123</v>
+      </c>
+      <c r="E10" s="17">
+        <f t="shared" si="0"/>
+        <v>6.0677770698704538E-2</v>
+      </c>
+      <c r="F10">
+        <v>139.32449999999997</v>
+      </c>
+      <c r="G10">
+        <v>169.27029872884989</v>
+      </c>
+      <c r="H10" s="17">
+        <v>0.9393222293012955</v>
+      </c>
+      <c r="I10">
+        <v>148.32449999999997</v>
+      </c>
+      <c r="J10">
+        <v>80.640352733603535</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11">
+        <v>13</v>
+      </c>
+      <c r="C11">
+        <v>13.923</v>
+      </c>
+      <c r="D11">
+        <v>5.5277782155220363</v>
+      </c>
+      <c r="E11" s="17">
+        <f t="shared" si="0"/>
+        <v>0.10589000308018758</v>
+      </c>
+      <c r="F11">
+        <v>117.56249999999999</v>
+      </c>
+      <c r="G11">
+        <v>135.47635792799363</v>
+      </c>
+      <c r="H11" s="17">
+        <v>0.89410999691981252</v>
+      </c>
+      <c r="I11">
+        <v>131.48549999999997</v>
+      </c>
+      <c r="J11">
+        <v>42.270848784948711</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>19.248000000000001</v>
+      </c>
+      <c r="D12">
+        <v>4.3842595726074425</v>
+      </c>
+      <c r="E12" s="17">
+        <f t="shared" si="0"/>
+        <v>0.32237966033564464</v>
+      </c>
+      <c r="F12">
+        <v>40.457999999999998</v>
+      </c>
+      <c r="G12">
+        <v>45.639963350492998</v>
+      </c>
+      <c r="H12" s="17">
+        <v>0.67762033966435531</v>
+      </c>
+      <c r="I12">
+        <v>59.706000000000003</v>
+      </c>
+      <c r="J12">
+        <v>9.2305958637565766</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13">
+        <v>13</v>
+      </c>
+      <c r="C13">
+        <v>21.72</v>
+      </c>
+      <c r="D13">
+        <v>11.202629869811819</v>
+      </c>
+      <c r="E13" s="17">
+        <f t="shared" si="0"/>
+        <v>0.32112126319524525</v>
+      </c>
+      <c r="F13">
+        <v>45.917999999999999</v>
+      </c>
+      <c r="G13">
+        <v>44.085153747196372</v>
+      </c>
+      <c r="H13" s="17">
+        <v>0.67887873680475463</v>
+      </c>
+      <c r="I13">
+        <v>67.638000000000005</v>
+      </c>
+      <c r="J13">
+        <v>2.500661512480248</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>19</v>
+      </c>
+      <c r="C14">
+        <v>34.571999999999996</v>
+      </c>
+      <c r="D14">
+        <v>22.194265205228131</v>
+      </c>
+      <c r="E14" s="17">
+        <f t="shared" si="0"/>
+        <v>0.51961403192352784</v>
+      </c>
+      <c r="F14">
+        <v>31.962</v>
+      </c>
+      <c r="G14">
+        <v>20.697659977192963</v>
+      </c>
+      <c r="H14" s="17">
+        <v>0.48038596807647221</v>
+      </c>
+      <c r="I14">
+        <v>66.533999999999992</v>
+      </c>
+      <c r="J14">
+        <v>23.62243586085059</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15">
+        <v>7</v>
+      </c>
+      <c r="C15">
+        <v>4.1340000000000003</v>
+      </c>
+      <c r="D15">
+        <v>3.8627653306925076</v>
+      </c>
+      <c r="E15" s="17">
+        <f t="shared" si="0"/>
+        <v>6.1391784727791152E-2</v>
+      </c>
+      <c r="F15">
+        <v>63.203999999999986</v>
+      </c>
+      <c r="G15">
+        <v>83.749710507659259</v>
+      </c>
+      <c r="H15" s="17">
+        <v>0.93860821527220872</v>
+      </c>
+      <c r="I15">
+        <v>67.337999999999994</v>
+      </c>
+      <c r="J15">
+        <v>40.613269604896381</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16">
+        <v>13</v>
+      </c>
+      <c r="C16">
+        <v>26.595000000000002</v>
+      </c>
+      <c r="D16">
+        <v>36.236394108685815</v>
+      </c>
+      <c r="E16" s="17">
+        <f t="shared" si="0"/>
+        <v>0.24179690696342365</v>
+      </c>
+      <c r="F16">
+        <v>83.393999999999991</v>
+      </c>
+      <c r="G16">
+        <v>89.419619697251093</v>
+      </c>
+      <c r="H16" s="17">
+        <v>0.7582030930365764</v>
+      </c>
+      <c r="I16">
+        <v>109.98899999999999</v>
+      </c>
+      <c r="J16">
+        <v>23.33028113846893</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17">
+        <v>19</v>
+      </c>
+      <c r="C17">
+        <v>8.8739999999999988</v>
+      </c>
+      <c r="D17">
+        <v>6.4912402512925054</v>
+      </c>
+      <c r="E17" s="17">
+        <f t="shared" si="0"/>
+        <v>0.10797196671046869</v>
+      </c>
+      <c r="F17">
+        <v>73.313999999999993</v>
+      </c>
+      <c r="G17">
+        <v>96.952796189006136</v>
+      </c>
+      <c r="H17" s="17">
+        <v>0.8920280332895314</v>
+      </c>
+      <c r="I17">
+        <v>82.187999999999988</v>
+      </c>
+      <c r="J17">
+        <v>15.171683097138567</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18">
+        <v>12</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>2.6279999999999997</v>
+      </c>
+      <c r="G18">
+        <v>2.6279999999999997</v>
+      </c>
+      <c r="H18" s="17">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>2.6279999999999997</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>